<commit_message>
docs: update Pythia-26 submission checklist with accurate status
- Fill GitHub repo URL
- Correct BlueVerse integration: No → Yes (backend/ai/blueverse.py)
- Correct caching: pickle → ChromaDB + sentence-transformers (RAG)
- Correct Oracle family: Peoplesoft → Oracle Fusion Cloud (HCM/ERP/OIC/BIP)
- Honest note on Dockerfile (deferred — render.yaml deploy instead)
- Honest note on multi-tenancy (scale-up path documented, not yet built)
- Honest note on Fusion REST hooks (OCI GenAI done; Fusion REST future)
- Fix Data sources: N/a → Yes (docs/LIMITATIONS.md §3-4)
- Tick 43 completed items across sections 1–7

Outstanding items are user-action-only:
- Demo video backup recording
- Team role assignment
- Submission email, demo slot, backup contact

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Pythia_Submission_Checklist.xlsx
+++ b/Pythia_Submission_Checklist.xlsx
@@ -546,7 +546,11 @@
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="5" t="inlineStr"/>
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
           <t>Onedrive/Sharepoint/GitHub/GitLab repository</t>
@@ -554,7 +558,7 @@
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>https://github.com/&lt;your-org&gt;/&lt;your-repo&gt;</t>
+          <t>https://github.com/Sameet1308/OracleImpactanalysisgenerator</t>
         </is>
       </c>
       <c r="D12" s="7" t="inlineStr">
@@ -564,7 +568,11 @@
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">
-      <c r="A13" s="5" t="inlineStr"/>
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
           <t>README.md file with project overview</t>
@@ -582,7 +590,11 @@
       </c>
     </row>
     <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="5" t="inlineStr"/>
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
           <t>Setup/Installation instructions in README</t>
@@ -600,7 +612,11 @@
       </c>
     </row>
     <row r="15" ht="22" customHeight="1">
-      <c r="A15" s="5" t="inlineStr"/>
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
           <t>Requirements.txt / package.json / dependencies file</t>
@@ -618,7 +634,11 @@
       </c>
     </row>
     <row r="16" ht="22" customHeight="1">
-      <c r="A16" s="5" t="inlineStr"/>
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
           <t>Environment variables template (.env.example)</t>
@@ -636,7 +656,11 @@
       </c>
     </row>
     <row r="17" ht="22" customHeight="1">
-      <c r="A17" s="5" t="inlineStr"/>
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
           <t>Code is well-commented and organized</t>
@@ -654,7 +678,11 @@
       </c>
     </row>
     <row r="18" ht="22" customHeight="1">
-      <c r="A18" s="5" t="inlineStr"/>
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
           <t>Architecture diagram (PNG/PDF)</t>
@@ -672,7 +700,11 @@
       </c>
     </row>
     <row r="19" ht="22" customHeight="1">
-      <c r="A19" s="5" t="inlineStr"/>
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
           <t>.gitignore file to exclude sensitive data</t>
@@ -719,7 +751,11 @@
       </c>
     </row>
     <row r="23" ht="22" customHeight="1">
-      <c r="A23" s="5" t="inlineStr"/>
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
           <t>BlueVerse API integration implemented</t>
@@ -727,7 +763,7 @@
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes — backend/ai/blueverse.py (BlueVerse Foundry JWT client, runtime token refresh, usage tracking)</t>
         </is>
       </c>
       <c r="D23" s="7" t="inlineStr">
@@ -737,7 +773,11 @@
       </c>
     </row>
     <row r="24" ht="22" customHeight="1">
-      <c r="A24" s="5" t="inlineStr"/>
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="B24" s="6" t="inlineStr">
         <is>
           <t>Fallback chain documented (BlueVerse → Claude → OpenAI/Gemini)</t>
@@ -755,7 +795,11 @@
       </c>
     </row>
     <row r="25" ht="22" customHeight="1">
-      <c r="A25" s="5" t="inlineStr"/>
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
           <t>Token usage logging implemented</t>
@@ -773,7 +817,11 @@
       </c>
     </row>
     <row r="26" ht="22" customHeight="1">
-      <c r="A26" s="5" t="inlineStr"/>
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="B26" s="6" t="inlineStr">
         <is>
           <t>Cost tracking per interaction</t>
@@ -791,7 +839,11 @@
       </c>
     </row>
     <row r="27" ht="22" customHeight="1">
-      <c r="A27" s="5" t="inlineStr"/>
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="B27" s="6" t="inlineStr">
         <is>
           <t>Prompt engineering strategy documented</t>
@@ -809,7 +861,11 @@
       </c>
     </row>
     <row r="28" ht="22" customHeight="1">
-      <c r="A28" s="5" t="inlineStr"/>
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="B28" s="6" t="inlineStr">
         <is>
           <t>Context management / caching strategy</t>
@@ -817,7 +873,7 @@
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
-          <t>pickle file strategy</t>
+          <t>ChromaDB + sentence-transformers (in-memory RAG, top-k retrieval) — backend/knowledge/rag.py</t>
         </is>
       </c>
       <c r="D28" s="7" t="inlineStr">
@@ -827,7 +883,11 @@
       </c>
     </row>
     <row r="29" ht="22" customHeight="1">
-      <c r="A29" s="5" t="inlineStr"/>
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
           <t>Multi-turn conversation handling</t>
@@ -874,7 +934,11 @@
       </c>
     </row>
     <row r="33" ht="22" customHeight="1">
-      <c r="A33" s="5" t="inlineStr"/>
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="B33" s="6" t="inlineStr">
         <is>
           <t>Oracle Product Family Contextualized</t>
@@ -882,7 +946,7 @@
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>Peoplesoft</t>
+          <t>Oracle Fusion Cloud (HCM, ERP, OIC, BIP) — parsers cover SQL/PL-SQL, OIC XML, BIP XML, Groovy</t>
         </is>
       </c>
       <c r="D33" s="7" t="inlineStr">
@@ -892,7 +956,11 @@
       </c>
     </row>
     <row r="34" ht="22" customHeight="1">
-      <c r="A34" s="5" t="inlineStr"/>
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="B34" s="6" t="inlineStr">
         <is>
           <t>RAG pipeline for Oracle documentation</t>
@@ -910,7 +978,11 @@
       </c>
     </row>
     <row r="35" ht="22" customHeight="1">
-      <c r="A35" s="5" t="inlineStr"/>
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
           <t>Provisions to add more Oracle context</t>
@@ -928,7 +1000,11 @@
       </c>
     </row>
     <row r="36" ht="22" customHeight="1">
-      <c r="A36" s="5" t="inlineStr"/>
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="B36" s="6" t="inlineStr">
         <is>
           <t>Oracle-specific terminology and workflows</t>
@@ -954,7 +1030,7 @@
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
-          <t>Fusion REST, JDE Orchestrations, etc.</t>
+          <t>OCI GenAI integrated; Fusion REST / JDE hooks scoped as future work</t>
         </is>
       </c>
       <c r="D37" s="7" t="inlineStr">
@@ -964,7 +1040,11 @@
       </c>
     </row>
     <row r="38" ht="22" customHeight="1">
-      <c r="A38" s="5" t="inlineStr"/>
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="B38" s="6" t="inlineStr">
         <is>
           <t>Cross-module adaptability demonstrated</t>
@@ -1011,7 +1091,11 @@
       </c>
     </row>
     <row r="42" ht="22" customHeight="1">
-      <c r="A42" s="5" t="inlineStr"/>
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="B42" s="6" t="inlineStr">
         <is>
           <t>Functional test cases documented</t>
@@ -1029,7 +1113,11 @@
       </c>
     </row>
     <row r="43" ht="22" customHeight="1">
-      <c r="A43" s="5" t="inlineStr"/>
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="B43" s="6" t="inlineStr">
         <is>
           <t>Edge case testing completed</t>
@@ -1047,7 +1135,11 @@
       </c>
     </row>
     <row r="44" ht="22" customHeight="1">
-      <c r="A44" s="5" t="inlineStr"/>
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="B44" s="6" t="inlineStr">
         <is>
           <t>Accuracy verification results</t>
@@ -1065,7 +1157,11 @@
       </c>
     </row>
     <row r="45" ht="22" customHeight="1">
-      <c r="A45" s="5" t="inlineStr"/>
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="B45" s="6" t="inlineStr">
         <is>
           <t>Performance benchmarks documented</t>
@@ -1083,7 +1179,11 @@
       </c>
     </row>
     <row r="46" ht="22" customHeight="1">
-      <c r="A46" s="5" t="inlineStr"/>
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="B46" s="6" t="inlineStr">
         <is>
           <t>Token usage optimization evidence</t>
@@ -1101,7 +1201,11 @@
       </c>
     </row>
     <row r="47" ht="22" customHeight="1">
-      <c r="A47" s="5" t="inlineStr"/>
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="B47" s="6" t="inlineStr">
         <is>
           <t>Error handling tested and documented</t>
@@ -1119,7 +1223,11 @@
       </c>
     </row>
     <row r="48" ht="22" customHeight="1">
-      <c r="A48" s="5" t="inlineStr"/>
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="B48" s="6" t="inlineStr">
         <is>
           <t>Multi-turn conversation testing</t>
@@ -1137,7 +1245,11 @@
       </c>
     </row>
     <row r="49" ht="22" customHeight="1">
-      <c r="A49" s="5" t="inlineStr"/>
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="B49" s="6" t="inlineStr">
         <is>
           <t>Cost comparison across LLM providers</t>
@@ -1184,7 +1296,11 @@
       </c>
     </row>
     <row r="53" ht="22" customHeight="1">
-      <c r="A53" s="5" t="inlineStr"/>
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="B53" s="6" t="inlineStr">
         <is>
           <t>Deployment instructions provided</t>
@@ -1210,7 +1326,7 @@
       </c>
       <c r="C54" s="6" t="inlineStr">
         <is>
-          <t>Dockerfile and docker-compose.yml</t>
+          <t>render.yaml deploy config (Render.com); Dockerfile deferred — container-clean design documented in docs/DEPLOYMENT.md §8</t>
         </is>
       </c>
       <c r="D54" s="7" t="inlineStr">
@@ -1220,7 +1336,11 @@
       </c>
     </row>
     <row r="55" ht="22" customHeight="1">
-      <c r="A55" s="5" t="inlineStr"/>
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="B55" s="6" t="inlineStr">
         <is>
           <t>Environment-specific configuration</t>
@@ -1238,7 +1358,11 @@
       </c>
     </row>
     <row r="56" ht="22" customHeight="1">
-      <c r="A56" s="5" t="inlineStr"/>
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="B56" s="6" t="inlineStr">
         <is>
           <t>Scalability considerations documented</t>
@@ -1264,7 +1388,7 @@
       </c>
       <c r="C57" s="6" t="inlineStr">
         <is>
-          <t>Client-specific customization capability</t>
+          <t>Scale-up path documented (tenant namespacing, per-tenant ChromaDB) — docs/DEPLOYMENT.md §5</t>
         </is>
       </c>
       <c r="D57" s="7" t="inlineStr">
@@ -1292,7 +1416,11 @@
       </c>
     </row>
     <row r="59" ht="22" customHeight="1">
-      <c r="A59" s="5" t="inlineStr"/>
+      <c r="A59" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="B59" s="6" t="inlineStr">
         <is>
           <t>Monitoring/logging strategy</t>
@@ -1339,7 +1467,11 @@
       </c>
     </row>
     <row r="63" ht="22" customHeight="1">
-      <c r="A63" s="5" t="inlineStr"/>
+      <c r="A63" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="B63" s="6" t="inlineStr">
         <is>
           <t>10-minute demo script prepared</t>
@@ -1357,7 +1489,11 @@
       </c>
     </row>
     <row r="64" ht="22" customHeight="1">
-      <c r="A64" s="5" t="inlineStr"/>
+      <c r="A64" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="B64" s="6" t="inlineStr">
         <is>
           <t>Working prototype deployed and accessible</t>
@@ -1393,7 +1529,11 @@
       </c>
     </row>
     <row r="66" ht="22" customHeight="1">
-      <c r="A66" s="5" t="inlineStr"/>
+      <c r="A66" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="B66" s="6" t="inlineStr">
         <is>
           <t>Use case KPI results prepared</t>
@@ -1411,7 +1551,11 @@
       </c>
     </row>
     <row r="67" ht="22" customHeight="1">
-      <c r="A67" s="5" t="inlineStr"/>
+      <c r="A67" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="B67" s="6" t="inlineStr">
         <is>
           <t>Q&amp;A preparation</t>
@@ -1429,7 +1573,11 @@
       </c>
     </row>
     <row r="68" ht="22" customHeight="1">
-      <c r="A68" s="5" t="inlineStr"/>
+      <c r="A68" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="B68" s="6" t="inlineStr">
         <is>
           <t>Demo data/scenarios ready</t>
@@ -1494,7 +1642,11 @@
       </c>
     </row>
     <row r="73" ht="22" customHeight="1">
-      <c r="A73" s="5" t="inlineStr"/>
+      <c r="A73" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="B73" s="6" t="inlineStr">
         <is>
           <t>Design document (2-5 pages)</t>
@@ -1512,7 +1664,11 @@
       </c>
     </row>
     <row r="74" ht="22" customHeight="1">
-      <c r="A74" s="5" t="inlineStr"/>
+      <c r="A74" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="B74" s="6" t="inlineStr">
         <is>
           <t>API documentation (if applicable)</t>
@@ -1530,7 +1686,11 @@
       </c>
     </row>
     <row r="75" ht="22" customHeight="1">
-      <c r="A75" s="5" t="inlineStr"/>
+      <c r="A75" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="B75" s="6" t="inlineStr">
         <is>
           <t>User guide or walkthrough</t>
@@ -1548,7 +1708,11 @@
       </c>
     </row>
     <row r="76" ht="22" customHeight="1">
-      <c r="A76" s="5" t="inlineStr"/>
+      <c r="A76" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="B76" s="6" t="inlineStr">
         <is>
           <t>Known limitations documented</t>
@@ -1566,7 +1730,11 @@
       </c>
     </row>
     <row r="77" ht="22" customHeight="1">
-      <c r="A77" s="5" t="inlineStr"/>
+      <c r="A77" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="B77" s="6" t="inlineStr">
         <is>
           <t>Data sources and assumptions documented</t>
@@ -1574,7 +1742,7 @@
       </c>
       <c r="C77" s="6" t="inlineStr">
         <is>
-          <t>N/a</t>
+          <t>Yes — docs/LIMITATIONS.md §3-4 (data sources, licensing, assumptions)</t>
         </is>
       </c>
       <c r="D77" s="7" t="inlineStr">
@@ -1584,7 +1752,11 @@
       </c>
     </row>
     <row r="78" ht="22" customHeight="1">
-      <c r="A78" s="5" t="inlineStr"/>
+      <c r="A78" s="5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="B78" s="6" t="inlineStr">
         <is>
           <t>Team member contributions documented</t>
@@ -1771,9 +1943,9 @@
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="A94:D94"/>
+    <mergeCell ref="A40:D40"/>
     <mergeCell ref="A80:D80"/>
-    <mergeCell ref="A40:D40"/>
-    <mergeCell ref="A94:D94"/>
     <mergeCell ref="A31:D31"/>
     <mergeCell ref="A8:D8"/>
     <mergeCell ref="A61:D61"/>

</xml_diff>